<commit_message>
Update mated assembly with physical caliper clearances: H17a (16.79mm back-of-box offset) and H17b (9.10mm vertical gap off plate)
</commit_message>
<xml_diff>
--- a/caliper_measurements.xlsx
+++ b/caliper_measurements.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caliper Measurements" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,50 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="000284C7"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00166534"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -76,41 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,2298 +413,2484 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="81" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Feature Description</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>How to Measure with Calipers</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Est. Range (mm)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Measured Value (mm)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Engineering Notes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Panel A: Plug Mating Face</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>[A1]</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Shroud Outer Width</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Widest outer horizontal span across orange oval shroud (exclude side key ribs)</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>36 - 38</t>
         </is>
       </c>
-      <c r="G2" s="5" t="n">
-        <v>36.1</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>36.1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Included tab</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Panel A: Plug Mating Face</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>[A2]</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Shroud Body Height</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Outer vertical height of oval body (bottom wall to arch below tower)</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>24 - 26</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>20.8</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Measured directly across oval</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Panel A: Plug Mating Face</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>[A3]</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Tower Outer Width</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Outer horizontal width across the top rectangular latch tower</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>14 - 16</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n">
-        <v>19.06</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>19.06</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Tower channel alignment</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Panel A: Plug Mating Face</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>[A4]</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Total Plug Height</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Bottom outer wall of oval shroud to top flat face of latch tower</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>34 - 36</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n">
-        <v>37.11</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>37.11</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Included tab (rib)</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Panel A: Plug Mating Face</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>[A5]</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Shroud Wall Thickness</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Caliper inside-to-outside thickness of orange outer perimeter wall</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>1.5 - 2.0</t>
         </is>
       </c>
-      <c r="G6" s="5" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>Internal clearance step</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Panel A: Plug Mating Face</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>[A6]</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Key Rib Protrusion</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Distance the side alignment keying rib sticks out from outer oval wall</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>2.0 - 2.5</t>
         </is>
       </c>
-      <c r="G7" s="5" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Slot keyway relief</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Panel B: Latch Tower &amp; Slider</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>[B1]</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Tower Axial Length</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Length of top rectangular tower from front mating rim back to shoulder/tape</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>18 - 22</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n">
-        <v>36.75</v>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>36.75</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Slide carriage base length</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Panel B: Latch Tower &amp; Slider</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>[B2]</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Slider Track Inner Width</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Inside width of channel/cavity where orange slider sits</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>10 - 12</t>
         </is>
       </c>
-      <c r="G9" s="5" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>17.8</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>Internal channel width</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Panel B: Latch Tower &amp; Slider</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>[B3]</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Slider Track Stroke Length</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Usable linear stroke length of yellow slider track</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>8 - 12</t>
         </is>
       </c>
-      <c r="G10" s="5" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>8.25</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>Slide travel range</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Panel B: Latch Tower &amp; Slider</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>[B4]</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Slider Total Length</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Overall length of detached orange slider piece</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>15 - 18</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n">
-        <v>23</v>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>23.0</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>CPA slider replacement ref</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Panel B: Latch Tower &amp; Slider</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>[B5]</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Slider Width</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Width across main body / thumb pad of orange slider</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>8 - 10</t>
         </is>
       </c>
-      <c r="G12" s="5" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>CPA slider replacement ref</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Panel B: Latch Tower &amp; Slider</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>[B6]</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Slider Thickness</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Thickness / height of orange slider piece</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>3 - 4</t>
         </is>
       </c>
-      <c r="G13" s="5" t="n">
-        <v>4.45</v>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>4.45</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>CPA slider replacement ref</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Panel B: Latch Tower &amp; Slider</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>[B7]</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Body Rigid Length</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Length of rigid orange housing from front rim to rear cable exit boot</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>45 - 55</t>
         </is>
       </c>
-      <c r="G14" s="5" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>54.6</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>Defines rear shoulder position where keeper locks</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Panel C: Outlet Receptacle</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>[C1]</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Collar Protrusion Length</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>How far black receptacle collar extends outward from black backplate</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>15 - 20</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n">
-        <v>22.37</v>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>22.37</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>Mating engagement depth</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Panel C: Outlet Receptacle</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>[C2]</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Tooth Distance from Rim</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Distance from front mating rim of black collar to vertical latch tooth step</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
         <is>
           <t>8 - 11</t>
         </is>
       </c>
-      <c r="G16" s="5" t="n">
-        <v>8.73</v>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>8.73</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>From farthest part of tooth which is sloped</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Panel C: Outlet Receptacle</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>[C3]</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Latch Tooth Width</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Width of raised latch tooth / ramp</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
         <is>
           <t>3 - 5</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>Locking tongue engagement</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Panel C: Outlet Receptacle</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>[C4]</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Latch Tooth Height</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Height latch tooth protrudes above outer top surface of collar</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>1.5 - 2.5</t>
         </is>
       </c>
-      <c r="G18" s="5" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>Max height, since tooth is sloped</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Panel C: Guide Ribs Spacing</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>[C5]</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Guide Ribs Spacing</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Outside width across the two guide ribs flanking the latch tooth</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>8 - 10</t>
         </is>
       </c>
-      <c r="G19" s="5" t="n">
-        <v>13.82</v>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>13.82</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>Exterior dimension</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Panel D: Receptacle Face &amp; Clearances</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>[D1]</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Collar Outer Width</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Horizontal outer width across black protruding receptacle collar</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>32 - 34</t>
         </is>
       </c>
-      <c r="G20" s="5" t="n">
-        <v>22.7</v>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>22.7</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>Includes alignment rib</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Panel D: Receptacle Face &amp; Clearances</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>[D2]</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Collar Outer Height</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Vertical outer height across black protruding receptacle collar</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>20 - 22</t>
         </is>
       </c>
-      <c r="G21" s="5" t="n">
-        <v>33.05</v>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>33.05</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>Includes alignment rib</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Panel D: Receptacle Face &amp; Clearances</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>[D3]</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Metal Plate Clearance</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Distance from right edge of black collar to vertical silver metal plate</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>6 - 9</t>
         </is>
       </c>
-      <c r="G22" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>Rough estimate</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Panel D: Receptacle Face &amp; Clearances</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>[D4]</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Top Clearance</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Free clearance above collar before hitting upper housing / wiring</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>10 - 15</t>
         </is>
       </c>
-      <c r="G23" s="5" t="n">
-        <v>8.27</v>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>8.27</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>Measured from top of enclosure to top of outer receptacle</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Panel E: Outlet Box Housing</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>[E1]</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Box Height</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Collar seating face up to top flat surface of the lid</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>38 - 44</t>
         </is>
       </c>
-      <c r="G24" s="5" t="n">
-        <v>42.67</v>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>42.67</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>Note: back of box is not flat where connector plugs in</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Panel E: Outlet Box Housing</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>[E2]</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Box Depth</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Front vertical wall to rear vertical wall across box body</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
         <is>
           <t>45 - 52</t>
         </is>
       </c>
-      <c r="G25" s="5" t="n">
-        <v>48.15</v>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>48.15</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
         <is>
           <t>Distance from front face to rear hook anchor</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Panel E: Outlet Box Housing</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>[E3a]</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Lid Overhang Height</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Vertical thickness / height of the overhanging lid rim</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
         <is>
           <t>3.0 - 5.0</t>
         </is>
       </c>
-      <c r="G26" s="5" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>4.58</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
         <is>
           <t>C-Spine hook drop height</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Panel E: Outlet Box Housing</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>[E3b]</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Lid Overhang Width</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Horizontal distance the lid lip extends past the rear wall</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t>8.0 - 15.0</t>
         </is>
       </c>
-      <c r="G27" s="5" t="n">
-        <v>12.45</v>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>12.45</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
         <is>
           <t>C-Spine hook shelf width (massive positive engagement)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Panel E: Outlet Box Housing</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>[E4]</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Box Width</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Width across the black housing section</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>48 - 56</t>
         </is>
       </c>
-      <c r="G28" s="5" t="n">
-        <v>49.65</v>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>49.65</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>Determines C-Spine interior clearance width (51.5mm)</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Panel E: Outlet Box Housing</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>[GAP]</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Seated Gap</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Distance between front face of connector and outlet housing when seated</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
         <is>
           <t>4.0 - 6.0</t>
         </is>
       </c>
-      <c r="G29" s="5" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
         <is>
           <t>Front connector clearance</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>[H1]</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Total Outer Width</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Widest horizontal span across outer housing edges</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
         <is>
           <t>140 - 180</t>
         </is>
       </c>
-      <c r="G30" s="5" t="n">
-        <v>142.3</v>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>142.3</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>[H2]</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Total Outer Height</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Bottom of lower chin to top outer rim face</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>90 - 100</t>
         </is>
       </c>
-      <c r="G31" s="5" t="n">
-        <v>95.40000000000001</v>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>[H3]</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Window Aperture Width</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Inside horizontal opening where AC outlet sits</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
         <is>
           <t>112 - 125</t>
         </is>
       </c>
-      <c r="G32" s="5" t="n">
-        <v>114.6</v>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>114.6</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
         <is>
           <t>Confirmed caliper (&gt;111.75mm outlet box)</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>[H4]</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Window Aperture Height</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Inside vertical height of rectangular opening</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
         <is>
           <t>48 - 58</t>
         </is>
       </c>
-      <c r="G33" s="5" t="n">
-        <v>50.2</v>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>50.2</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>[H5]</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Lower Chin Height</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Vertical thickness of protruding bottom bar</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>25 - 32</t>
         </is>
       </c>
-      <c r="G34" s="5" t="n">
-        <v>30.77</v>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>30.77</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>[H5b]</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Chin Total Thickness</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Front-to-back depth of chin including molded ribs in back</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
         <is>
           <t>6.0 - 8.5</t>
         </is>
       </c>
-      <c r="G35" s="5" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>Confirmed caliper (user refined)</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>[H6]</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Top Bezel Frame Thickness</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Distance from top outer rim to top of window aperture</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>8 - 14</t>
         </is>
       </c>
-      <c r="G36" s="5" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
         <is>
           <t>Calculated from 95.40 - 84.20</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>[H7a]</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Side Wall Depth</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Front bezel face straight back to rear plastic edge of side wing</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
         <is>
           <t>55 - 65</t>
         </is>
       </c>
-      <c r="G37" s="5" t="n">
-        <v>58.8</v>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>58.8</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>[H9]</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Top Shelf Flat Length</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Length of horizontal top section before angled drop</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>30 - 40</t>
         </is>
       </c>
-      <c r="G38" s="5" t="n">
-        <v>34</v>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>[H10]</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Aluminum Rear Extension</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Distance silver sheet metal clip extends backwards</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>45 - 55</t>
         </is>
       </c>
-      <c r="G39" s="5" t="n">
-        <v>53</v>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>[H11]</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Inner Wing Clear Span</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Clear inside width between left and right side walls</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
         <is>
           <t>135 - 145</t>
         </is>
       </c>
-      <c r="G40" s="5" t="n">
-        <v>140.5</v>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>140.5</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>[H11b]</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Wing to Aluminum Space</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>Horizontal clearance between plastic wing and horizontal aluminum plate</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
         <is>
           <t>9.0 - 11.5</t>
         </is>
       </c>
-      <c r="G41" s="5" t="n">
-        <v>10.15</v>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>10.15</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
         <is>
           <t>Confirmed caliper (user refined)</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>[H12]</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Aluminum Bracket Width</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>Width of horizontal stamped sheet metal frame</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
         <is>
           <t>118 - 125</t>
         </is>
       </c>
-      <c r="G42" s="5" t="n">
-        <v>120.2</v>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>120.2</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
         <is>
           <t>140.50 - 2x10.15 = 120.20mm</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>[H13]</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Side Wall Thickness</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>Plastic wall thickness of the side wings</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>2.0 - 3.0</t>
         </is>
       </c>
-      <c r="G43" s="5" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>[H14]</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Window Recess Step Depth</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Depth of internal ledge where outlet face seats</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>2.5 - 4.0</t>
         </is>
       </c>
-      <c r="G44" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>[H15a]</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Aluminum Outer Hole Offset</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Distance from side of aluminum to outer edge of horizontal oval slot</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
         <is>
           <t>14 - 18</t>
         </is>
       </c>
-      <c r="G45" s="5" t="n">
-        <v>16.75</v>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>16.75</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>[H15b]</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>Aluminum Outer Oval Width (X)</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>Width of horizontal oval slot along X (rotated 90 deg)</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
         <is>
           <t>6.5 - 8.5</t>
         </is>
       </c>
-      <c r="G46" s="5" t="n">
-        <v>7.45</v>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>7.45</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
         <is>
           <t>Confirmed caliper (horizontal slot)</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>[H15c]</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Aluminum Holes Edge Spacing</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Distance from inner edge of oval slot to outer edge of central hole</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
         <is>
           <t>35 - 40</t>
         </is>
       </c>
-      <c r="G47" s="5" t="n">
-        <v>37.95</v>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>37.95</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>[H15d]</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Aluminum Central Hole Diameter</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Diameter of central circular round hole through aluminum floor</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
         <is>
           <t>5.5 - 7.5</t>
         </is>
       </c>
-      <c r="G48" s="5" t="n">
-        <v>6.45</v>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>6.45</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
         <is>
           <t>Confirmed caliper</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="2" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>[H15e]</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>Aluminum Holes Center Spacing</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Center-to-center distance between the two holes</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
         <is>
           <t>40 - 50</t>
         </is>
       </c>
-      <c r="G49" s="5" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>44.9</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
         <is>
           <t>Calculated center-to-center</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>[H15f]</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>Central Hole Back Edge Dist</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>Distance from back edge of aluminum to central hole</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
         <is>
           <t>6.0 - 9.0</t>
         </is>
       </c>
-      <c r="G50" s="5" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>7.6</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
         <is>
           <t>Confirmed caliper (7.6mm to back edge)</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>[H15g]</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Outer Oval Back Edge Dist</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Distance from back edge of aluminum to outer horizontal oval slot</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
         <is>
           <t>6.0 - 9.0</t>
         </is>
       </c>
-      <c r="G51" s="5" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
         <is>
           <t>Confirmed caliper (7.3mm to back edge)</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>[H16a]</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>50mm Triangle Chord Distance</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>Distance between 50mm marks on traced angle legs</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
         <is>
           <t>64 - 70</t>
         </is>
       </c>
-      <c r="G52" s="5" t="n">
-        <v>67</v>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>67.0</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
         <is>
           <t>Confirmed caliper (chord C=67mm)</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="2" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>[H16b]</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>Internal Bend Angle</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>Calibrated internal bend angle of aluminum plate</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
         <is>
           <t>82 - 86</t>
         </is>
       </c>
-      <c r="G53" s="5" t="n">
-        <v>84.13</v>
-      </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>84.13</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
         <is>
           <t>2 * arcsin(67/100) = 84.13 deg</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>[H16c]</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>Upward Pitch Angle</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>Upward tilt angle of aluminum plate toward ceiling</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
         <is>
           <t>4.0 - 8.0</t>
         </is>
       </c>
-      <c r="G54" s="5" t="n">
-        <v>5.87</v>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>5.87</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
         <is>
           <t>90.0 - 84.13 = 5.87 deg pitch</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="2" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>[H16d]</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>Wing Bottom Termination</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>Vertical height where side wings terminate (aligned with window)</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
         <is>
           <t>32 - 36</t>
         </is>
       </c>
-      <c r="G55" s="5" t="n">
-        <v>34</v>
-      </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>34.0</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
         <is>
           <t>Aligned with window bottom</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>[H16f]</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Chin Below Aluminum Plate</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>Vertical distance chin extends down below aluminum plate</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
         <is>
           <t>25 - 29</t>
         </is>
       </c>
-      <c r="G56" s="5" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>27.1</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
         <is>
           <t>Confirmed caliper (chin extends 27.1mm)</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="inlineStr">
         <is>
           <t>Panel F: Outer Housing Bezel</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>[H16g]</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>Plate Below Window Aperture</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>Vertical distance aluminum plate is below window opening</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
         <is>
           <t>6.0 - 8.0</t>
         </is>
       </c>
-      <c r="G57" s="5" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>6.9</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
         <is>
           <t>Confirmed caliper (plate 6.9mm below window)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Panel F: Outer Housing Bezel</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>[H17a]</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Back of Box to Back of Plate</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Horizontal distance from back of aluminum plate forward to back wall of outlet box</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>15 - 18</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>16.79</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Leaves 16.79mm of rear plate clear so chassis bolt holes are completely uncovered</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Panel F: Outer Housing Bezel</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>[H17b]</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Box Vertical Gap off Plate</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Vertical clearance between bottom surface of outlet box and near horizontal aluminum plate</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>8 - 10</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Bottom of box sits ~9.1mm above aluminum plate (2.2mm above window bottom sill)</t>
         </is>
       </c>
     </row>

</xml_diff>